<commit_message>
removed comp calc V1 from excel sheet
</commit_message>
<xml_diff>
--- a/Battery Charger Project/Excel/Calculations/Component calcs.xlsx
+++ b/Battery Charger Project/Excel/Calculations/Component calcs.xlsx
@@ -8,15 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Verrazano\Acedemic\Research\Battery-Charger\Battery Charger Project\Excel\Calculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6DF3313-3E1C-4ED8-9B3C-2A9C410F5E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD1EA3CA-0187-40E0-B44F-10DD8DCC7EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{8EA801AC-1218-4C2A-8BFC-BC5B39F04A2A}"/>
+    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{8EA801AC-1218-4C2A-8BFC-BC5B39F04A2A}"/>
   </bookViews>
   <sheets>
-    <sheet name="24V analysis V2" sheetId="1" r:id="rId1"/>
-    <sheet name="12V analysis V2" sheetId="2" r:id="rId2"/>
-    <sheet name="24V analysis V1" sheetId="4" r:id="rId3"/>
-    <sheet name="12V analysis V1" sheetId="5" r:id="rId4"/>
+    <sheet name="24V analysis" sheetId="1" r:id="rId1"/>
+    <sheet name="12V analysis" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -42,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="65">
   <si>
     <t>C-rate</t>
   </si>
@@ -2079,7 +2077,7 @@
         <v>64</v>
       </c>
       <c r="N5" s="7">
-        <f>'24V analysis V2'!N6</f>
+        <f>'24V analysis'!N6</f>
         <v>6.5886173588108662E-5</v>
       </c>
       <c r="O5" s="8" t="s">
@@ -2338,1111 +2336,6 @@
       <c r="F21" s="13">
         <f>F18*F20</f>
         <v>1.5427784316797402</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="E22" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F22" s="13">
-        <f>F19*F20</f>
-        <v>21.6</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="E23" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F23" s="13">
-        <v>500</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A24" s="21"/>
-      <c r="B24" s="21"/>
-      <c r="C24" s="21"/>
-      <c r="E24" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="F24" s="13">
-        <v>0.3</v>
-      </c>
-      <c r="G24" s="5"/>
-    </row>
-    <row r="25" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="E25" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="F25" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="G25" s="5"/>
-    </row>
-    <row r="26" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="E26" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="F26" s="13">
-        <f>F24*F20</f>
-        <v>7.1999999999999993</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E27" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="F27" s="14">
-        <f>F25*F17</f>
-        <v>0.14599999999999999</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="E13:G13"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A603C2-9CB9-4EDD-96B4-465A647A4A00}">
-  <dimension ref="A1:R28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.109375" customWidth="1"/>
-    <col min="17" max="17" width="13" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="24"/>
-      <c r="E1" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="19"/>
-      <c r="G1" s="20"/>
-      <c r="I1" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="J1" s="19"/>
-      <c r="K1" s="20"/>
-      <c r="M1" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="N1" s="19"/>
-      <c r="O1" s="20"/>
-    </row>
-    <row r="2" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" s="13">
-        <f>F4/SQRT(2)</f>
-        <v>24.024478110041532</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" s="13">
-        <f>F17/F19</f>
-        <v>32.444444444444443</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="N2" s="17">
-        <f>((F17*(1-(F17/F15)))/(F26*F23*10^3))</f>
-        <v>6.5167593819901747E-6</v>
-      </c>
-      <c r="O2" s="16" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>8</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="13">
-        <v>110</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" s="13">
-        <f>((3/PI())*F5)</f>
-        <v>148.55219216592252</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="N3">
-        <f>((F19*F14)*(1-F19))/(F26*F23*10^3)</f>
-        <v>8.1111111111111105E-7</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <f>B2*B3</f>
-        <v>24</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="13">
-        <f>((PI()/3)*J2)</f>
-        <v>33.975742772156281</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="J4" s="13">
-        <f>B18</f>
-        <v>480</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="N4">
-        <f>(((1-F18)*B20)/(2*F23*10^3))</f>
-        <v>7.2113931974347563E-7</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>2.5</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="13">
-        <f>SQRT(2)*F3</f>
-        <v>155.56349186104046</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="J5" s="13">
-        <f>B19</f>
-        <v>700.8</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="N5">
-        <f>((1-('12V analysis V1'!F18))/(8*N2*F25*(F23*10^3)^2))</f>
-        <v>7.1560382789616669E-6</v>
-      </c>
-      <c r="O5" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="R5" s="11"/>
-    </row>
-    <row r="6" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="7">
-        <v>3.65</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F6" s="13">
-        <f>SQRT(2/3)*J6</f>
-        <v>2.6382536207043161</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J6" s="13">
-        <f>F21</f>
-        <v>3.231187591387902</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="N6" s="7">
-        <f>N2</f>
-        <v>6.5167593819901747E-6</v>
-      </c>
-      <c r="O6" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="13">
-        <f>SQRT(2/3)*J7</f>
-        <v>17.636326148038883</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="J7" s="14">
-        <f>F22</f>
-        <v>21.6</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="E8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="13">
-        <f>SQRT(3)*F6*F3</f>
-        <v>502.65482457436673</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E9" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="14">
-        <f>SQRT(3)*F2*F7</f>
-        <v>733.8760438785755</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="M10" s="13"/>
-    </row>
-    <row r="12" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="23"/>
-      <c r="C13" s="24"/>
-      <c r="E13" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="F13" s="19"/>
-      <c r="G13" s="20"/>
-    </row>
-    <row r="14" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" s="2">
-        <v>24</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F14" s="13">
-        <f>J2</f>
-        <v>32.444444444444443</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15">
-        <v>8</v>
-      </c>
-      <c r="C15" s="5"/>
-      <c r="E15" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F15" s="13">
-        <f>J3</f>
-        <v>148.55219216592252</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16">
-        <f>B5*B15</f>
-        <v>20</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F16" s="13">
-        <f>B16</f>
-        <v>20</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17">
-        <f>B6*B15</f>
-        <v>29.2</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" s="13">
-        <f>B17</f>
-        <v>29.2</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B18">
-        <f>B16*B4</f>
-        <v>480</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F18" s="13">
-        <f>F16/J3</f>
-        <v>0.13463281630782925</v>
-      </c>
-      <c r="G18" s="5"/>
-    </row>
-    <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19">
-        <f>B17*B4</f>
-        <v>700.8</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F19" s="13">
-        <v>0.9</v>
-      </c>
-      <c r="G19" s="5"/>
-    </row>
-    <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B20" s="13">
-        <f>B16/B4</f>
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F20" s="13">
-        <v>24</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" s="14">
-        <f>B17/B4</f>
-        <v>1.2166666666666666</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" s="13">
-        <f>F18*F20</f>
-        <v>3.231187591387902</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="E22" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F22" s="13">
-        <f>F19*F20</f>
-        <v>21.6</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="E23" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F23" s="13">
-        <v>500</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A24" s="21"/>
-      <c r="B24" s="21"/>
-      <c r="C24" s="21"/>
-      <c r="E24" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="F24" s="13">
-        <v>0.3</v>
-      </c>
-      <c r="G24" s="5"/>
-    </row>
-    <row r="25" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="E25" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="F25" s="13">
-        <v>0.01</v>
-      </c>
-      <c r="G25" s="5"/>
-    </row>
-    <row r="26" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="E26" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F26" s="13">
-        <f>F24*F20</f>
-        <v>7.1999999999999993</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="E27" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F27" s="13">
-        <f>F25*F17</f>
-        <v>0.29199999999999998</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E28" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F28" s="7">
-        <f>SQRT(((F20^2)+(3.6^2)))</f>
-        <v>24.268498099388022</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="E1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0420058C-2B98-43A8-B8E2-0DAD44F0257E}">
-  <dimension ref="A1:O27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="4.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="24"/>
-      <c r="E1" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" s="19"/>
-      <c r="G1" s="20"/>
-      <c r="I1" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="J1" s="19"/>
-      <c r="K1" s="20"/>
-      <c r="M1" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="N1" s="19"/>
-      <c r="O1" s="20"/>
-    </row>
-    <row r="2" spans="1:15" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" s="13">
-        <f>F4/SQRT(2)</f>
-        <v>12.012239055020766</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" s="13">
-        <f>F17/F19</f>
-        <v>16.222222222222221</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="N2">
-        <f>((F17*(1-(F17/F15)))/(F26*F23*10^3))</f>
-        <v>3.6569676232753216E-6</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>8</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="13">
-        <v>110</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" s="13">
-        <f>((3/PI())*F5)</f>
-        <v>148.55219216592252</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="N3">
-        <f>((F19*F14)*(1-F19))/(F26*F23*10^3)</f>
-        <v>4.0555555555555553E-7</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <f>B2*B3</f>
-        <v>24</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="13">
-        <f>((PI()/3)*J2)</f>
-        <v>16.98787138607814</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="J4" s="13">
-        <f>B18</f>
-        <v>240</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="N4">
-        <f>(((1-F18)*B20)/(2*F23*10^3))</f>
-        <v>3.8861816326920227E-7</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>2.5</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="13">
-        <f>SQRT(2)*F3</f>
-        <v>155.56349186104046</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="J5" s="13">
-        <f>B19</f>
-        <v>350.4</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="N5" s="7">
-        <f>'24V analysis V1'!N6</f>
-        <v>6.5167593819901747E-6</v>
-      </c>
-      <c r="O5" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="7">
-        <v>3.65</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F6" s="13">
-        <f>SQRT(2/3)*J6</f>
-        <v>1.3191268103521581</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J6" s="13">
-        <f>F21</f>
-        <v>1.615593795693951</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="13">
-        <f>SQRT(2/3)*J7</f>
-        <v>17.636326148038883</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="J7" s="14">
-        <f>F22</f>
-        <v>21.6</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="E8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="13">
-        <f>SQRT(3)*F6*F3</f>
-        <v>251.32741228718336</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="E9" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="14">
-        <f>SQRT(3)*F2*F7</f>
-        <v>366.93802193928775</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H9" s="12"/>
-    </row>
-    <row r="12" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="13" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="23"/>
-      <c r="C13" s="24"/>
-      <c r="E13" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="F13" s="19"/>
-      <c r="G13" s="20"/>
-    </row>
-    <row r="14" spans="1:15" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" s="2">
-        <v>12</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F14" s="13">
-        <f>J2</f>
-        <v>16.222222222222221</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15">
-        <v>4</v>
-      </c>
-      <c r="C15" s="5"/>
-      <c r="E15" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F15" s="13">
-        <f>J3</f>
-        <v>148.55219216592252</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16">
-        <f>B5*B15</f>
-        <v>10</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F16" s="13">
-        <f>B16</f>
-        <v>10</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17">
-        <f>B6*B15</f>
-        <v>14.6</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" s="13">
-        <f>B17</f>
-        <v>14.6</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B18">
-        <f>B16*B4</f>
-        <v>240</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F18" s="13">
-        <f>F16/J3</f>
-        <v>6.7316408153914625E-2</v>
-      </c>
-      <c r="G18" s="5"/>
-    </row>
-    <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19">
-        <f>B17*B4</f>
-        <v>350.4</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F19" s="13">
-        <v>0.9</v>
-      </c>
-      <c r="G19" s="5"/>
-    </row>
-    <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B20" s="13">
-        <f>B16/B4</f>
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F20" s="13">
-        <v>24</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" s="14">
-        <f>B17/B4</f>
-        <v>0.60833333333333328</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" s="13">
-        <f>F18*F20</f>
-        <v>1.615593795693951</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>30</v>
@@ -3531,6 +2424,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="77b6129a-f613-4ff9-b238-21504ab3c311" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009660838691862E40BA8A9FCF4672D404" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="57f0f8c66996a8cfd8079b5f5cbc1044">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="77b6129a-f613-4ff9-b238-21504ab3c311" xmlns:ns4="e5775723-78a2-49b3-980c-6ad0b4b03e58" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="97be24bc9c367c471a14e5d43da4af43" ns3:_="" ns4:_="">
     <xsd:import namespace="77b6129a-f613-4ff9-b238-21504ab3c311"/>
@@ -3719,38 +2629,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="77b6129a-f613-4ff9-b238-21504ab3c311" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F510E196-854A-4018-94EA-77433BC9C36C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D69E919-C42D-4F67-B937-7A9547F9358A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="77b6129a-f613-4ff9-b238-21504ab3c311"/>
-    <ds:schemaRef ds:uri="e5775723-78a2-49b3-980c-6ad0b4b03e58"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3773,9 +2655,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D69E919-C42D-4F67-B937-7A9547F9358A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F510E196-854A-4018-94EA-77433BC9C36C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="77b6129a-f613-4ff9-b238-21504ab3c311"/>
+    <ds:schemaRef ds:uri="e5775723-78a2-49b3-980c-6ad0b4b03e58"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated sim and clacs
I changed the charging current from 3C (24A) to 1C (8A). I updated the simulation graphs and calculations.
</commit_message>
<xml_diff>
--- a/Battery Charger Project/Excel/Calculations/Component calcs.xlsx
+++ b/Battery Charger Project/Excel/Calculations/Component calcs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Verrazano\Acedemic\Research\Battery-Charger\Battery Charger Project\Excel\Calculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBD8F7CB-AF91-4034-9EF8-A66BC5E94E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F6444C-A616-496B-93D5-209210E97215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{8EA801AC-1218-4C2A-8BFC-BC5B39F04A2A}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{8EA801AC-1218-4C2A-8BFC-BC5B39F04A2A}"/>
   </bookViews>
   <sheets>
     <sheet name="24V analysis" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="68">
   <si>
     <t>C-rate</t>
   </si>
@@ -976,7 +976,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1023,9 +1023,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1361,21 +1360,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CAB43F6-C991-4FED-A486-EADAA5F16055}">
   <dimension ref="A1:R26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.88671875" customWidth="1"/>
-    <col min="7" max="7" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.21875" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.28515625" customWidth="1"/>
     <col min="17" max="17" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
         <v>17</v>
       </c>
@@ -1397,12 +1396,12 @@
       <c r="N1" s="26"/>
       <c r="O1" s="27"/>
     </row>
-    <row r="2" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
-        <v>3</v>
+      <c r="B2" s="32">
+        <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>2</v>
@@ -1432,17 +1431,17 @@
       </c>
       <c r="N2" s="20">
         <f>((F17*(1-(F17/F15)))/(F26*F23*10^3))</f>
-        <v>6.5886173588108662E-5</v>
+        <v>1.9765852076432595E-4</v>
       </c>
       <c r="O2" s="16" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:18" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="32">
         <v>8</v>
       </c>
       <c r="C3" s="5" t="s">
@@ -1472,19 +1471,19 @@
       </c>
       <c r="N3" s="7">
         <f>((1-(F18))/(8*N2*F25*(F23*10^3)^2))</f>
-        <v>6.6131866766249291E-5</v>
+        <v>2.1929478272464733E-5</v>
       </c>
       <c r="O3" s="8" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="32">
         <f>B2*B3</f>
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>4</v>
@@ -1503,18 +1502,18 @@
       </c>
       <c r="J4" s="21">
         <f>B18</f>
-        <v>480</v>
+        <v>165.63200000000001</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B5">
-        <v>2.5</v>
+      <c r="B5" s="32">
+        <v>2.5880000000000001</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>7</v>
@@ -1534,21 +1533,21 @@
       </c>
       <c r="J5" s="21">
         <f>B19</f>
-        <v>700.8</v>
+        <v>233.6</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>16</v>
       </c>
       <c r="R5" s="11"/>
     </row>
-    <row r="6" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:18" ht="18" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="32">
         <v>3.65</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E6" s="4" t="s">
@@ -1556,7 +1555,7 @@
       </c>
       <c r="F6" s="21">
         <f>SQRT(2/3)*J6</f>
-        <v>2.5193466291910944</v>
+        <v>0.86934254351287354</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>30</v>
@@ -1566,20 +1565,20 @@
       </c>
       <c r="J6" s="21">
         <f>F21</f>
-        <v>3.0855568633594803</v>
+        <v>1.0647228216499112</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="32" t="s">
+    <row r="7" spans="1:18" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="33">
-        <v>3.1</v>
-      </c>
-      <c r="C7" s="34" t="s">
+      <c r="B7" s="32">
+        <v>2.5</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="4" t="s">
@@ -1587,7 +1586,7 @@
       </c>
       <c r="F7" s="21">
         <f>SQRT(2/3)*J7</f>
-        <v>9.5366800652358403</v>
+        <v>3.1788933550786131</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>30</v>
@@ -1597,21 +1596,21 @@
       </c>
       <c r="J7" s="22">
         <f>F22</f>
-        <v>11.68</v>
+        <v>3.8933333333333331</v>
       </c>
       <c r="K7" s="8" t="s">
         <v>30</v>
       </c>
       <c r="M7" s="13"/>
     </row>
-    <row r="8" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A8" s="32" t="s">
+    <row r="8" spans="1:18" ht="18" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="33">
-        <v>3.45</v>
-      </c>
-      <c r="C8" s="34" t="s">
+      <c r="B8" s="32">
+        <v>3.5579999999999998</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E8" s="4" t="s">
@@ -1619,26 +1618,46 @@
       </c>
       <c r="F8" s="21">
         <f>SQRT(3)*F6*F3</f>
-        <v>479.99999999999994</v>
+        <v>165.63199999999998</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:18" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="33">
+        <v>7.6E-3</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>15</v>
+      </c>
       <c r="E9" s="6" t="s">
         <v>12</v>
       </c>
       <c r="F9" s="22">
         <f>SQRT(3)*F2*F7</f>
-        <v>700.8</v>
+        <v>233.59999999999997</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="22">
+        <v>1.14E-2</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="29" t="s">
         <v>18</v>
       </c>
@@ -1650,7 +1669,7 @@
       <c r="F13" s="26"/>
       <c r="G13" s="27"/>
     </row>
-    <row r="14" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
@@ -1674,7 +1693,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="18" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>10</v>
       </c>
@@ -1693,13 +1712,13 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" ht="18" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="B16" s="21">
         <f>B5*B15</f>
-        <v>20</v>
+        <v>20.704000000000001</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>7</v>
@@ -1709,15 +1728,15 @@
       </c>
       <c r="F16" s="21">
         <f>B16</f>
-        <v>20</v>
+        <v>20.704000000000001</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="B17" s="21">
         <f>B6*B15</f>
@@ -1737,13 +1756,13 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B18" s="21">
         <f>B16*B4</f>
-        <v>480</v>
+        <v>165.63200000000001</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>16</v>
@@ -1753,17 +1772,17 @@
       </c>
       <c r="F18" s="21">
         <f>F16/J3</f>
-        <v>0.12856486930664501</v>
+        <v>0.1330903527062389</v>
       </c>
       <c r="G18" s="5"/>
     </row>
-    <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B19" s="21">
         <f>B17*B4</f>
-        <v>700.8</v>
+        <v>233.6</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>16</v>
@@ -1777,12 +1796,13 @@
       </c>
       <c r="G19" s="5"/>
     </row>
-    <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B20" s="21">
-        <v>7.6E-3</v>
+        <f>B15*B9</f>
+        <v>6.08E-2</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>15</v>
@@ -1791,18 +1811,20 @@
         <v>29</v>
       </c>
       <c r="F20" s="21">
-        <v>24</v>
+        <f>B4</f>
+        <v>8</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="6" t="s">
         <v>14</v>
       </c>
       <c r="B21" s="22">
-        <v>1.2E-2</v>
+        <f>B15*B10</f>
+        <v>9.1200000000000003E-2</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>15</v>
@@ -1812,25 +1834,25 @@
       </c>
       <c r="F21" s="21">
         <f>F18*F20</f>
-        <v>3.0855568633594803</v>
+        <v>1.0647228216499112</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="E22" s="4" t="s">
         <v>38</v>
       </c>
       <c r="F22" s="21">
         <f>F19*F20</f>
-        <v>11.68</v>
+        <v>3.8933333333333331</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E23" s="4" t="s">
         <v>47</v>
       </c>
@@ -1841,7 +1863,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A24" s="28"/>
       <c r="B24" s="28"/>
       <c r="C24" s="28"/>
@@ -1853,7 +1875,7 @@
       </c>
       <c r="G24" s="5"/>
     </row>
-    <row r="25" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="E25" s="10" t="s">
         <v>54</v>
       </c>
@@ -1862,13 +1884,13 @@
       </c>
       <c r="G25" s="5"/>
     </row>
-    <row r="26" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E26" s="6" t="s">
         <v>55</v>
       </c>
       <c r="F26" s="22">
         <f>F24*F20</f>
-        <v>7.1999999999999993</v>
+        <v>2.4</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>30</v>
@@ -1892,18 +1914,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF31E89F-592A-437D-9440-200F7F48CEED}">
   <dimension ref="A1:P26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="4.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="2.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.88671875" customWidth="1"/>
+    <col min="16" max="16" width="6.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
         <v>17</v>
       </c>
@@ -1925,7 +1947,7 @@
       <c r="N1" s="26"/>
       <c r="O1" s="27"/>
     </row>
-    <row r="2" spans="1:16" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1966,7 +1988,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -2000,7 +2022,7 @@
       </c>
       <c r="N3" s="18">
         <f>((1-(F18))/(8*'24V analysis'!N2*F25*(F23*10^3)^2))</f>
-        <v>7.1010161494304677E-5</v>
+        <v>2.3670053831434897E-5</v>
       </c>
       <c r="O3" s="19" t="s">
         <v>58</v>
@@ -2009,7 +2031,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
@@ -2040,7 +2062,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
@@ -2071,7 +2093,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:16" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
@@ -2102,7 +2124,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:16" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E7" s="4" t="s">
         <v>42</v>
       </c>
@@ -2127,7 +2149,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="18" x14ac:dyDescent="0.35">
       <c r="E8" s="4" t="s">
         <v>11</v>
       </c>
@@ -2139,7 +2161,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:16" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E9" s="6" t="s">
         <v>12</v>
       </c>
@@ -2152,8 +2174,8 @@
       </c>
       <c r="H9" s="12"/>
     </row>
-    <row r="12" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="13" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="29" t="s">
         <v>19</v>
       </c>
@@ -2165,7 +2187,7 @@
       <c r="F13" s="26"/>
       <c r="G13" s="27"/>
     </row>
-    <row r="14" spans="1:16" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
@@ -2189,7 +2211,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" ht="18" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>10</v>
       </c>
@@ -2208,7 +2230,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" ht="18" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>8</v>
       </c>
@@ -2230,7 +2252,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>9</v>
       </c>
@@ -2252,7 +2274,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>11</v>
       </c>
@@ -2272,7 +2294,7 @@
       </c>
       <c r="G18" s="5"/>
     </row>
-    <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>12</v>
       </c>
@@ -2292,7 +2314,7 @@
       </c>
       <c r="G19" s="5"/>
     </row>
-    <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>13</v>
       </c>
@@ -2313,7 +2335,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="6" t="s">
         <v>14</v>
       </c>
@@ -2335,7 +2357,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="E22" s="4" t="s">
         <v>38</v>
       </c>
@@ -2347,7 +2369,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E23" s="4" t="s">
         <v>47</v>
       </c>
@@ -2358,7 +2380,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A24" s="28"/>
       <c r="B24" s="28"/>
       <c r="C24" s="28"/>
@@ -2370,7 +2392,7 @@
       </c>
       <c r="G24" s="5"/>
     </row>
-    <row r="25" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="E25" s="4" t="s">
         <v>51</v>
       </c>
@@ -2379,7 +2401,7 @@
       </c>
       <c r="G25" s="5"/>
     </row>
-    <row r="26" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E26" s="24" t="s">
         <v>53</v>
       </c>

</xml_diff>